<commit_message>
D2 the parameter sheet takes the group, data type and samples the IMC key read in Revit gives, group Text (Q336)
</commit_message>
<xml_diff>
--- a/config/shared_parameters.xlsx
+++ b/config/shared_parameters.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -505,7 +505,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2441</t>
+          <t>2391</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>VD2</t>
+          <t>VD1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>VD2-T1</t>
+          <t>VD1-T1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SCHEDULES OF VRF INDOOR &amp; OUTDOOR UNITS-VD2</t>
+          <t>SCHEDULES OF VRF INDOOR &amp; OUTDOOR UNITS-DP1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2441 | VD2 | 1 | XX | XX</t>
+          <t>2391 | VD1 | 1 | XX | XX</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -837,11 +837,6 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>7 Place villas</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>A</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -868,7 +863,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">

</xml_diff>